<commit_message>
Ajustes gerais + Readme
</commit_message>
<xml_diff>
--- a/amostras/controle/K04/matriz_rastreabilidade_K04.xlsx
+++ b/amostras/controle/K04/matriz_rastreabilidade_K04.xlsx
@@ -814,6 +814,7 @@
           <t>Nenhuma</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>Nenhum</t>
@@ -871,6 +872,7 @@
           <t>Nenhuma</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>Nenhum</t>
@@ -928,6 +930,7 @@
           <t>Nenhuma</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>Nenhum</t>
@@ -985,6 +988,7 @@
           <t>Nenhuma</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>Nenhum</t>
@@ -1042,6 +1046,7 @@
           <t>Nenhuma</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>Nenhum</t>
@@ -1099,6 +1104,7 @@
           <t>Nenhuma</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>Nenhum</t>
@@ -1156,6 +1162,7 @@
           <t>Nenhuma</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>Nenhum</t>
@@ -1213,6 +1220,7 @@
           <t>Nenhuma</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>Nenhum</t>
@@ -1270,6 +1278,7 @@
           <t>Nenhuma</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>Nenhum</t>
@@ -1327,6 +1336,7 @@
           <t>Nenhuma</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>Nenhum</t>
@@ -1384,6 +1394,7 @@
           <t>Nenhuma</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>Nenhum</t>
@@ -1441,6 +1452,7 @@
           <t>Nenhuma</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>Nenhum</t>
@@ -1498,6 +1510,7 @@
           <t>Nenhuma</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>Nenhum</t>
@@ -1555,6 +1568,7 @@
           <t>Nenhuma</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>Nenhum</t>
@@ -1612,6 +1626,7 @@
           <t>Nenhuma</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>Nenhum</t>

</xml_diff>